<commit_message>
Denetim duzeltmeleri (dusuk oncelik): yama araci kural tabanli liste, USB guncellemesi configs'i korur, kurulum sablonu nem/kojen rolleri, log saatleri, kullanilmayan kod ve eski dosyalar temizlendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yeni_lokasyon_kurulum_sablonu.xlsx
+++ b/yeni_lokasyon_kurulum_sablonu.xlsx
@@ -10,9 +10,10 @@
     <sheet name="Lokasyon Profili" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Modbus Analizorler" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="BACnet Noktalar" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AHU Noktalari" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="AHU SAT ve Kapasite" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Talimatlar" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Roller" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="AHU Noktalari" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="AHU SAT ve Kapasite" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Talimatlar" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -638,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1223,7 +1224,7 @@
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  6. CHILLER / FCU KAPASITE BILGISI (Opsiyonel — kojen/uretim hesabi icin)</t>
+          <t xml:space="preserve">  6. CHILLER / KAZAN / FCU KAPASITE BILGISI (Opsiyonel — talep/uretim hesabi icin)</t>
         </is>
       </c>
     </row>
@@ -1284,96 +1285,114 @@
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>FCU Adedi</t>
+          <t>Kazan Birim Kapasite (kW)</t>
         </is>
       </c>
       <c r="B47" s="5" t="n"/>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Toplam FCU sayisi</t>
+          <t>Tek bir kazanin kW isitma kapasitesi (adet: 17. satir)</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Ornek: 1750</t>
+          <t>Ornek: 1950</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>FCU Birim Kapasite (kW)</t>
+          <t>FCU Adedi</t>
         </is>
       </c>
       <c r="B48" s="5" t="n"/>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Tek bir FCU biriminin ortalama kW kapasitesi</t>
+          <t>Toplam FCU sayisi</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Ornek: 2.5</t>
+          <t>Ornek: 1750</t>
         </is>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>FCU Esanjor Diversity</t>
+          <t>FCU Birim Kapasite (kW)</t>
         </is>
       </c>
       <c r="B49" s="5" t="n"/>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Eszamanlilik faktoru (0-1 arasi)</t>
+          <t>Tek bir FCU biriminin ortalama kW kapasitesi</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Ornek: 0.55</t>
+          <t>Ornek: 2.5</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Tasarim Hava DT (C)</t>
+          <t>FCU Esanjor Diversity</t>
         </is>
       </c>
       <c r="B50" s="5" t="n"/>
       <c r="C50" s="6" t="inlineStr">
         <is>
+          <t>Eszamanlilik faktoru (0-1 arasi)</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Ornek: 0.55</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Tasarim Hava DT (C)</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
           <t>AHU/FCU tasarim hava sicaklik farki</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>Ornek: 5</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="8" customHeight="1"/>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="3" t="inlineStr">
+    <row r="52" ht="8" customHeight="1"/>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  7. LiSANS BiLGiSi (Lokasyon ID ile KARISTIRMAYIN — farkli kavramlar)</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Makine ID</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n"/>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Lokasyon PC sinin anakart UUID si — PC de "wmic csproduct get uuid" komutuyla alinir. Bu, Lokasyon ID DEGiLDiR, ayri bir kavramdir.</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>Ornek: DF9ABA0D-A7A8-C416-A430-00D861BD5794</t>
         </is>
@@ -1384,9 +1403,9 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A53:D53"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A11:D11"/>
@@ -2428,7 +2447,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="I4:I54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Dis Hava Sicakligi,Chiller Set Sicakligi,Hat1 Isitma Sicakligi,Hat1 Sogutma Sicakligi,Hat1 Kazan Sicakligi,Hat2 Isitma Sicakligi,Hat2 Sogutma Sicakligi,Hat2 Kazan Sicakligi,Chiller-1 Durum,Chiller-2 Durum,Chiller-3 Durum,Chiller-4 Durum,Chiller-5 Durum,Chiller-1 Yuzde,Chiller-2 Yuzde,Chiller-3 Yuzde,Chiller-4 Yuzde,Chiller-5 Yuzde,Absorpsiyon Chiller Durum,Kazan-1 Durum,Kazan-2 Durum,Kazan-3 Durum,Kullanilmayacak"</formula1>
+      <formula1>=Roller!$A$1:$A$28</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2436,6 +2455,216 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Dis Hava Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dis Hava Nem</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Chiller Set Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hat1 Isitma Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hat1 Sogutma Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hat1 Kazan Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hat2 Isitma Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hat2 Sogutma Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Hat2 Kazan Sicakligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Chiller-1 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Chiller-2 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Chiller-3 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Chiller-4 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Chiller-5 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Chiller-1 Yuzde</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Chiller-2 Yuzde</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Chiller-3 Yuzde</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Chiller-4 Yuzde</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Chiller-5 Yuzde</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Absorpsiyon Chiller Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Kazan-1 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Kazan-2 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Kazan-3 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Kojen-1 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Kojen-2 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Kojen-3 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Kojen-4 Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Kullanilmayacak</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3061,13 +3290,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3075,6 +3304,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3087,7 +3317,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>OPSiYONEL sayfa — doldurulmazsa sistem genel varsayilan degerlerle calisir. Her AHU icin ozel sogutma/isitma SAT (ufleme) limiti ve tasarim kapasitesi (kW) girilirse analiz daha dogru olur.</t>
+          <t>OPSiYONEL sayfa — doldurulmazsa sistem genel varsayilan degerlerle calisir. Her AHU icin ozel sogutma/isitma SAT (ufleme) limiti ve tasarim kapasiteleri (kW) girilirse analiz daha dogru olur. Sogutma ve isitma kapasiteleri, mekanik zeka ekranindaki talep-uretim kartlarinin hesabinda kullanilir.</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3344,12 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Tasarim Kapasitesi (kW)</t>
+          <t>Tasarim Sogutma Kapasitesi (kW)</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Tasarim Isitma Kapasitesi (kW)</t>
         </is>
       </c>
     </row>
@@ -3137,6 +3372,9 @@
       </c>
       <c r="E4" s="11" t="n">
         <v>194.9</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>182.2</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -3145,6 +3383,7 @@
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="n"/>
@@ -3152,6 +3391,7 @@
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="n"/>
@@ -3159,6 +3399,7 @@
       <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="5" t="n"/>
@@ -3166,6 +3407,7 @@
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="n"/>
@@ -3173,6 +3415,7 @@
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="n"/>
       <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="n"/>
@@ -3180,6 +3423,7 @@
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="n"/>
@@ -3187,6 +3431,7 @@
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="5" t="n"/>
@@ -3194,6 +3439,7 @@
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="n"/>
@@ -3201,6 +3447,7 @@
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="n"/>
       <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="5" t="n"/>
@@ -3208,6 +3455,7 @@
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="n"/>
@@ -3215,6 +3463,7 @@
       <c r="C15" s="5" t="n"/>
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="5" t="n"/>
@@ -3222,6 +3471,7 @@
       <c r="C16" s="5" t="n"/>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="5" t="n"/>
@@ -3229,6 +3479,7 @@
       <c r="C17" s="5" t="n"/>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="5" t="n"/>
@@ -3236,6 +3487,7 @@
       <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="n"/>
@@ -3243,6 +3495,7 @@
       <c r="C19" s="5" t="n"/>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="5" t="n"/>
@@ -3250,6 +3503,7 @@
       <c r="C20" s="5" t="n"/>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="5" t="n"/>
@@ -3257,6 +3511,7 @@
       <c r="C21" s="5" t="n"/>
       <c r="D21" s="5" t="n"/>
       <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="5" t="n"/>
@@ -3264,6 +3519,7 @@
       <c r="C22" s="5" t="n"/>
       <c r="D22" s="5" t="n"/>
       <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="5" t="n"/>
@@ -3271,6 +3527,7 @@
       <c r="C23" s="5" t="n"/>
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="5" t="n"/>
@@ -3278,6 +3535,7 @@
       <c r="C24" s="5" t="n"/>
       <c r="D24" s="5" t="n"/>
       <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="5" t="n"/>
@@ -3285,6 +3543,7 @@
       <c r="C25" s="5" t="n"/>
       <c r="D25" s="5" t="n"/>
       <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="5" t="n"/>
@@ -3292,6 +3551,7 @@
       <c r="C26" s="5" t="n"/>
       <c r="D26" s="5" t="n"/>
       <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="5" t="n"/>
@@ -3299,6 +3559,7 @@
       <c r="C27" s="5" t="n"/>
       <c r="D27" s="5" t="n"/>
       <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="5" t="n"/>
@@ -3306,6 +3567,7 @@
       <c r="C28" s="5" t="n"/>
       <c r="D28" s="5" t="n"/>
       <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="5" t="n"/>
@@ -3313,6 +3575,7 @@
       <c r="C29" s="5" t="n"/>
       <c r="D29" s="5" t="n"/>
       <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="5" t="n"/>
@@ -3320,6 +3583,7 @@
       <c r="C30" s="5" t="n"/>
       <c r="D30" s="5" t="n"/>
       <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="5" t="n"/>
@@ -3327,6 +3591,7 @@
       <c r="C31" s="5" t="n"/>
       <c r="D31" s="5" t="n"/>
       <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="5" t="n"/>
@@ -3334,6 +3599,7 @@
       <c r="C32" s="5" t="n"/>
       <c r="D32" s="5" t="n"/>
       <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="5" t="n"/>
@@ -3341,6 +3607,7 @@
       <c r="C33" s="5" t="n"/>
       <c r="D33" s="5" t="n"/>
       <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="5" t="n"/>
@@ -3348,6 +3615,7 @@
       <c r="C34" s="5" t="n"/>
       <c r="D34" s="5" t="n"/>
       <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
@@ -3358,15 +3626,15 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A35:F35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3498,7 +3766,7 @@
       <c r="A13" s="21" t="inlineStr"/>
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - ahu_sat_limitleri.json / ahu_tasarim_kapasiteleri.json  (AHU SAT ve Kapasite sayfasindan, doldurulduysa)</t>
+          <t xml:space="preserve">  - ahu_sat_limitleri.json / ahu_tasarim_kapasiteleri.json / ahu_tasarim_isitma_kapasiteleri.json  (AHU SAT ve Kapasite sayfasindan, doldurulduysa)</t>
         </is>
       </c>
     </row>

</xml_diff>